<commit_message>
Update UI tram dien tkvv
</commit_message>
<xml_diff>
--- a/public/TagTramDienTKVV.xlsx
+++ b/public/TagTramDienTKVV.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07C7341-DD2C-4186-94D9-1FE4604DF3AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6549743E-3D5E-4492-AFE0-C3ECDA915DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="599" firstSheet="2" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="2595" windowWidth="15150" windowHeight="11385" tabRatio="599" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TUDOLUONGDAUVAO_35KV" sheetId="30" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="217">
   <si>
     <t>Tag0</t>
   </si>
@@ -618,12 +618,6 @@
     <t>Lộ 1 Khử Khí Khói-HA11</t>
   </si>
   <si>
-    <t>Tủ đầu vào MBA T1 35/10kV-SB01</t>
-  </si>
-  <si>
-    <t>Tủ đầu vào MBA T2 35/10kV-SB02</t>
-  </si>
-  <si>
     <t>Tủ đầu vào TC 10kV lộ 2 - HB08</t>
   </si>
   <si>
@@ -670,6 +664,24 @@
   </si>
   <si>
     <t>°C</t>
+  </si>
+  <si>
+    <t>Điện Áp pha A</t>
+  </si>
+  <si>
+    <t>Điện Áp pha B</t>
+  </si>
+  <si>
+    <t>Điện Áp pha C</t>
+  </si>
+  <si>
+    <t>Tủ đầu vào MBA T1 35/10kV-SA01</t>
+  </si>
+  <si>
+    <t>Tủ đầu vào MBA T2 35/10kV-SB01</t>
+  </si>
+  <si>
+    <t>Cosphi</t>
   </si>
 </sst>
 </file>
@@ -817,6 +829,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -824,6 +841,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -841,14 +861,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1132,151 +1144,153 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" customWidth="1"/>
     <col min="3" max="3" width="22.42578125" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>183</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>211</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+        <v>32</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>212</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+        <v>33</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>213</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+        <v>34</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>178</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+        <v>36</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="18"/>
+        <v>37</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="10" t="s">
         <v>184</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>211</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+        <v>110</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>212</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+        <v>111</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+        <v>112</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>177</v>
       </c>
@@ -1284,14 +1298,14 @@
         <v>9</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>211</v>
+        <v>113</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>178</v>
       </c>
@@ -1299,25 +1313,25 @@
         <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>211</v>
+        <v>114</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="2" t="s">
+      <c r="A12" s="12"/>
+      <c r="B12" s="1" t="s">
         <v>179</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>211</v>
+        <v>115</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -1327,6 +1341,7 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1342,7 +1357,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>194</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1354,12 +1369,12 @@
       <c r="D1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1369,12 +1384,12 @@
       <c r="D2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -1384,12 +1399,12 @@
       <c r="D3" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1399,12 +1414,12 @@
       <c r="D4" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -1414,12 +1429,12 @@
       <c r="D5" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -1432,8 +1447,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>206</v>
+      <c r="A7" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -1444,12 +1459,12 @@
       <c r="D7" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1459,12 +1474,12 @@
       <c r="D8" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1474,12 +1489,12 @@
       <c r="D9" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -1489,12 +1504,12 @@
       <c r="D10" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -1504,12 +1519,12 @@
       <c r="D11" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -1519,7 +1534,7 @@
       <c r="D12" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
@@ -1548,7 +1563,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1560,12 +1575,12 @@
       <c r="D1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1575,12 +1590,12 @@
       <c r="D2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -1590,12 +1605,12 @@
       <c r="D3" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1605,12 +1620,12 @@
       <c r="D4" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -1620,12 +1635,12 @@
       <c r="D5" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -1638,8 +1653,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>205</v>
+      <c r="A7" s="10" t="s">
+        <v>203</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -1650,12 +1665,12 @@
       <c r="D7" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1665,12 +1680,12 @@
       <c r="D8" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1680,12 +1695,12 @@
       <c r="D9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -1695,12 +1710,12 @@
       <c r="D10" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -1710,12 +1725,12 @@
       <c r="D11" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -1725,7 +1740,7 @@
       <c r="D12" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1749,7 +1764,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>191</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1761,12 +1776,12 @@
       <c r="D1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1776,12 +1791,12 @@
       <c r="D2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -1791,12 +1806,12 @@
       <c r="D3" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1806,12 +1821,12 @@
       <c r="D4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -1821,12 +1836,12 @@
       <c r="D5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
+      <c r="A6" s="11"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -1839,8 +1854,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>202</v>
+      <c r="A7" s="10" t="s">
+        <v>200</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -1851,12 +1866,12 @@
       <c r="D7" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1866,12 +1881,12 @@
       <c r="D8" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -1881,12 +1896,12 @@
       <c r="D9" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -1896,12 +1911,12 @@
       <c r="D10" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -1911,12 +1926,12 @@
       <c r="D11" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -1926,7 +1941,7 @@
       <c r="D12" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1939,7 +1954,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BAB0F4C-8F8B-407B-94A9-D6D54F46933C}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
@@ -1949,7 +1964,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="13" t="s">
         <v>185</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1961,12 +1976,12 @@
       <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="13"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1976,12 +1991,12 @@
       <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="13"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -1991,12 +2006,12 @@
       <c r="D3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -2006,12 +2021,12 @@
       <c r="D4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -2021,12 +2036,12 @@
       <c r="D5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -2036,192 +2051,102 @@
       <c r="D6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="17"/>
+      <c r="E6" s="8"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="2" t="s">
-        <v>25</v>
+      <c r="A7" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>212</v>
+        <v>116</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
+      <c r="A8" s="13"/>
+      <c r="B8" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>212</v>
+        <v>117</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="2" t="s">
-        <v>24</v>
+      <c r="A9" s="13"/>
+      <c r="B9" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>212</v>
+        <v>118</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>197</v>
-      </c>
+      <c r="A10" s="13"/>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>208</v>
+        <v>119</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>176</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-      <c r="B13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E15" s="17"/>
-    </row>
-    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
-      <c r="B18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>212</v>
-      </c>
+      <c r="E12" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:A9"/>
-    <mergeCell ref="A10:A18"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="A7:A12"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2241,7 +2166,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="14" t="s">
         <v>186</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -2253,12 +2178,12 @@
       <c r="D1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
+      <c r="A2" s="15"/>
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
@@ -2268,12 +2193,12 @@
       <c r="D2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
+      <c r="A3" s="15"/>
       <c r="B3" s="2" t="s">
         <v>20</v>
       </c>
@@ -2283,12 +2208,12 @@
       <c r="D3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="11"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
@@ -2298,12 +2223,12 @@
       <c r="D4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
@@ -2313,12 +2238,12 @@
       <c r="D5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
+      <c r="A6" s="16"/>
       <c r="B6" s="2" t="s">
         <v>176</v>
       </c>
@@ -2331,7 +2256,7 @@
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="17" t="s">
         <v>187</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -2343,12 +2268,12 @@
       <c r="D7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>211</v>
+      <c r="E7" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="2" t="s">
         <v>181</v>
       </c>
@@ -2358,12 +2283,12 @@
       <c r="D8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>211</v>
+      <c r="E8" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="18"/>
       <c r="B9" s="2" t="s">
         <v>182</v>
       </c>
@@ -2373,13 +2298,13 @@
       <c r="D9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>211</v>
+      <c r="E9" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>198</v>
+      <c r="A10" s="14" t="s">
+        <v>196</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>180</v>
@@ -2390,12 +2315,12 @@
       <c r="D10" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>211</v>
+      <c r="E10" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
+      <c r="A11" s="15"/>
       <c r="B11" s="2" t="s">
         <v>181</v>
       </c>
@@ -2405,12 +2330,12 @@
       <c r="D11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>211</v>
+      <c r="E11" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="2" t="s">
         <v>182</v>
       </c>
@@ -2420,8 +2345,8 @@
       <c r="D12" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="16" t="s">
-        <v>211</v>
+      <c r="E12" s="7" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -2437,7 +2362,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59791292-26F9-4C6C-A09B-6FC2A2D62802}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -2447,8 +2372,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>195</v>
+      <c r="A1" s="13" t="s">
+        <v>214</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -2456,182 +2381,274 @@
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="D1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="13"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="D2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="13"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="D3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="D4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="13"/>
+      <c r="B6" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="13"/>
+      <c r="B7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
+      <c r="B8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="13"/>
+      <c r="B9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="13"/>
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="13"/>
+      <c r="B12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="13"/>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="13"/>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E14" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="13"/>
+      <c r="B15" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="13"/>
+      <c r="B16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E6" s="18"/>
-    </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" s="16" t="s">
+    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="13"/>
+      <c r="B17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E12" s="18"/>
+    <row r="18" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>210</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:A6"/>
-    <mergeCell ref="A7:A12"/>
+    <mergeCell ref="A1:A9"/>
+    <mergeCell ref="A10:A18"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2647,8 +2664,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>207</v>
+      <c r="A1" s="10" t="s">
+        <v>205</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -2659,12 +2676,12 @@
       <c r="D1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -2674,12 +2691,12 @@
       <c r="D2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -2689,12 +2706,12 @@
       <c r="D3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -2704,12 +2721,12 @@
       <c r="D4" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -2719,12 +2736,12 @@
       <c r="D5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -2737,8 +2754,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>204</v>
+      <c r="A7" s="10" t="s">
+        <v>202</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -2749,12 +2766,12 @@
       <c r="D7" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -2764,12 +2781,12 @@
       <c r="D8" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -2779,12 +2796,12 @@
       <c r="D9" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -2794,12 +2811,12 @@
       <c r="D10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -2809,12 +2826,12 @@
       <c r="D11" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -2824,7 +2841,7 @@
       <c r="D12" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2847,7 +2864,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>188</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2859,12 +2876,12 @@
       <c r="D1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -2874,12 +2891,12 @@
       <c r="D2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -2889,12 +2906,12 @@
       <c r="D3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -2904,12 +2921,12 @@
       <c r="D4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -2919,12 +2936,12 @@
       <c r="D5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -2937,8 +2954,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>199</v>
+      <c r="A7" s="10" t="s">
+        <v>197</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -2949,12 +2966,12 @@
       <c r="D7" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -2964,12 +2981,12 @@
       <c r="D8" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -2979,12 +2996,12 @@
       <c r="D9" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -2994,12 +3011,12 @@
       <c r="D10" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -3009,12 +3026,12 @@
       <c r="D11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -3024,7 +3041,7 @@
       <c r="D12" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3048,7 +3065,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3060,12 +3077,12 @@
       <c r="D1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -3075,12 +3092,12 @@
       <c r="D2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -3090,12 +3107,12 @@
       <c r="D3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -3105,12 +3122,12 @@
       <c r="D4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -3120,12 +3137,12 @@
       <c r="D5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -3138,8 +3155,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>200</v>
+      <c r="A7" s="10" t="s">
+        <v>198</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -3150,12 +3167,12 @@
       <c r="D7" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -3165,12 +3182,12 @@
       <c r="D8" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -3180,12 +3197,12 @@
       <c r="D9" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -3195,12 +3212,12 @@
       <c r="D10" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -3210,12 +3227,12 @@
       <c r="D11" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -3225,7 +3242,7 @@
       <c r="D12" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3249,7 +3266,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>190</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3261,12 +3278,12 @@
       <c r="D1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -3276,12 +3293,12 @@
       <c r="D2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -3291,12 +3308,12 @@
       <c r="D3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -3306,12 +3323,12 @@
       <c r="D4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -3321,12 +3338,12 @@
       <c r="D5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -3339,8 +3356,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>201</v>
+      <c r="A7" s="10" t="s">
+        <v>199</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -3351,12 +3368,12 @@
       <c r="D7" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -3366,12 +3383,12 @@
       <c r="D8" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -3381,12 +3398,12 @@
       <c r="D9" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -3396,12 +3413,12 @@
       <c r="D10" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -3411,12 +3428,12 @@
       <c r="D11" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -3426,7 +3443,7 @@
       <c r="D12" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3449,7 +3466,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>192</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -3461,12 +3478,12 @@
       <c r="D1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="16" t="s">
-        <v>208</v>
+      <c r="E1" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
@@ -3476,12 +3493,12 @@
       <c r="D2" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="16" t="s">
-        <v>208</v>
+      <c r="E2" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>20</v>
       </c>
@@ -3491,12 +3508,12 @@
       <c r="D3" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E3" s="16" t="s">
-        <v>208</v>
+      <c r="E3" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -3506,12 +3523,12 @@
       <c r="D4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>209</v>
+      <c r="E4" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
@@ -3521,12 +3538,12 @@
       <c r="D5" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>210</v>
+      <c r="E5" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
+      <c r="A6" s="12"/>
       <c r="B6" s="1" t="s">
         <v>176</v>
       </c>
@@ -3539,8 +3556,8 @@
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>203</v>
+      <c r="A7" s="10" t="s">
+        <v>201</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
@@ -3551,12 +3568,12 @@
       <c r="D7" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E7" s="16" t="s">
-        <v>208</v>
+      <c r="E7" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
@@ -3566,12 +3583,12 @@
       <c r="D8" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="E8" s="16" t="s">
-        <v>208</v>
+      <c r="E8" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>20</v>
       </c>
@@ -3581,12 +3598,12 @@
       <c r="D9" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E9" s="16" t="s">
-        <v>208</v>
+      <c r="E9" s="7" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="11"/>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
@@ -3596,12 +3613,12 @@
       <c r="D10" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>209</v>
+      <c r="E10" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
+      <c r="A11" s="11"/>
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -3611,12 +3628,12 @@
       <c r="D11" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>210</v>
+      <c r="E11" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="1" t="s">
         <v>176</v>
       </c>
@@ -3626,7 +3643,7 @@
       <c r="D12" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E12" s="18"/>
+      <c r="E12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>